<commit_message>
paper run 2026-10-20 16:41
</commit_message>
<xml_diff>
--- a/reports/2026-10-20.xlsx
+++ b/reports/2026-10-20.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,178 @@
         <is>
           <t>P&amp;L $</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-20T11:43:58.078753+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="G2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.769</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-0.00104</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>3.96</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-20T15:39:02.932259+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F3" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="G3" t="n">
+        <v>60</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.00121</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>-34.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-20T15:53:45.890876+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F4" t="n">
+        <v>60.43</v>
+      </c>
+      <c r="G4" t="n">
+        <v>102.42</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00133</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>41.99</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-20T16:27:44.353655+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F5" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>90</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00125</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>34.2</v>
       </c>
     </row>
   </sheetData>
@@ -485,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +679,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +689,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -527,7 +699,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -536,6 +708,9 @@
           <t>winrate</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,7 +719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>45.35</v>
       </c>
     </row>
     <row r="7">
@@ -554,7 +729,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>80.15000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -564,7 +739,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-34.8</v>
       </c>
     </row>
     <row r="9">
@@ -573,6 +748,9 @@
           <t>pf</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>2.3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,7 +759,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3574.409999999999</v>
+        <v>3619.759999999999</v>
       </c>
     </row>
     <row r="12">
@@ -628,161 +806,594 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1261.47</v>
+      </c>
+      <c r="E15" t="n">
+        <v>34.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>11</v>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" t="n">
+        <v>426.73</v>
+      </c>
+      <c r="E16" t="n">
+        <v>11.15</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>По активам</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>123.71</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-0.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" t="n">
+        <v>7</v>
+      </c>
+      <c r="D19" t="n">
+        <v>674.14</v>
+      </c>
+      <c r="E19" t="n">
+        <v>41.99</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>9</v>
+      </c>
+      <c r="C20" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" t="n">
+        <v>890.35</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.96</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" t="n">
+        <v>265.5</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>9</v>
+      </c>
+      <c r="C23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" t="n">
+        <v>826.5599999999999</v>
+      </c>
+      <c r="E23" t="n">
+        <v>11.15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" t="n">
+        <v>596.14</v>
+      </c>
+      <c r="E24" t="n">
+        <v>34.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>260.22</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>15</v>
+      </c>
+      <c r="C27" t="n">
+        <v>13</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1253.65</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="n">
+        <v>174.33</v>
+      </c>
+      <c r="E28" t="n">
+        <v>45.35</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>41.99</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3.96</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>34.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="n">
+        <v>11.15</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>3.96</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>7.19</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>34.2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>11.15</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>34.2</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3.96</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="n">
+        <v>41.39</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>3.36</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>41.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-20 22:21
</commit_message>
<xml_diff>
--- a/reports/2026-10-20.xlsx
+++ b/reports/2026-10-20.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,49 +601,6 @@
       </c>
       <c r="K4" t="n">
         <v>41.99</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-10-20T16:27:44.353655+00:00</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>15</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="F5" t="n">
-        <v>55.8</v>
-      </c>
-      <c r="G5" t="n">
-        <v>90</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.792</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-0.00125</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>34.2</v>
       </c>
     </row>
   </sheetData>
@@ -657,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,7 +636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -689,7 +646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -709,7 +666,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.75</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="6">
@@ -719,7 +676,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>45.35</v>
+        <v>11.15</v>
       </c>
     </row>
     <row r="7">
@@ -729,7 +686,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>80.15000000000001</v>
+        <v>45.95</v>
       </c>
     </row>
     <row r="8">
@@ -749,7 +706,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.3</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="10">
@@ -759,7 +716,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3619.759999999999</v>
+        <v>3585.559999999999</v>
       </c>
     </row>
     <row r="12">
@@ -810,16 +767,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>1261.47</v>
+        <v>898.6</v>
       </c>
       <c r="E15" t="n">
-        <v>34.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -855,16 +812,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>123.71</v>
+        <v>21.06</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.6</v>
+        <v>-34.8</v>
       </c>
     </row>
     <row r="19">
@@ -874,13 +831,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" t="n">
-        <v>674.14</v>
+        <v>565.66</v>
       </c>
       <c r="E19" t="n">
         <v>41.99</v>
@@ -893,13 +850,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>890.35</v>
+        <v>738.61</v>
       </c>
       <c r="E20" t="n">
         <v>3.96</v>
@@ -919,13 +876,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>265.5</v>
+        <v>113.76</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -957,16 +914,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>596.14</v>
+        <v>385.01</v>
       </c>
       <c r="E24" t="n">
-        <v>34.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -979,17 +936,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
+          <t>NO_LIQUIDITY</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D26" t="n">
-        <v>260.22</v>
+        <v>1253.65</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -998,90 +955,87 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>1253.65</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>4</v>
-      </c>
-      <c r="C28" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" t="n">
-        <v>174.33</v>
-      </c>
-      <c r="E28" t="n">
-        <v>45.35</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+        <v>11.15</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-34.8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" t="n">
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.6</v>
+        <v>41.99</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1091,153 +1045,143 @@
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>41.99</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="n">
         <v>3.96</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
-        <v>34.2</v>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>11.15</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>3</v>
-      </c>
-      <c r="C39" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" t="n">
-        <v>11.15</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>3.96</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>3.96</v>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>7.19</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>2</v>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" t="n">
-        <v>7.19</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
-        <v>34.2</v>
+        <v>11.15</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По силе движения</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1259,39 +1203,39 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>11.15</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.12–0.15%</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" t="n">
         <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>34.2</v>
+        <v>7.19</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>По силе движения</t>
+          <t>По направлению</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1313,86 +1257,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C51" t="n">
         <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>3.96</v>
+        <v>-30.84</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>41.39</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>3</v>
-      </c>
-      <c r="C55" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" t="n">
-        <v>3.36</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" t="n">
         <v>41.99</v>
       </c>
     </row>

</xml_diff>